<commit_message>
Updated and new scripts
</commit_message>
<xml_diff>
--- a/SARIMA_Outputs/agriculture_cereal_best_auto_sarima_results.xlsx
+++ b/SARIMA_Outputs/agriculture_cereal_best_auto_sarima_results.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eskom-my.sharepoint.com/personal/mauduh_eskom_co_za/Documents/SARIMA_Outputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eskom-my.sharepoint.com/personal/mauduh_eskom_co_za/Documents/Python Projects/Parameter-Optimisation/SARIMA_Outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_3F155D949467860E62355476585DCE3A8747644A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCAD34C1-9600-487D-B988-A4A5F288DE93}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_3F155D949467860E62355476585DCE3A8747644A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{667717D6-8A6D-49A7-9F8F-659EBDDE92B6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$U$29</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -2364,6 +2367,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U29" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>